<commit_message>
delete note reg and add all code in adding....ipyn lets do the training
</commit_message>
<xml_diff>
--- a/labeled/june/without straw/Hydrocare_ffinal.xlsx
+++ b/labeled/june/without straw/Hydrocare_ffinal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alireza.mohammadshafie/Documents/hydrocare/labeled/june/without straw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBB94AAF-CE5E-4F4C-A93D-CD91AE7B02FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C8BB508-0A09-4042-A575-461ABC9778E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15100" yWindow="760" windowWidth="15140" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="33">
   <si>
     <t>ID</t>
   </si>
@@ -110,6 +110,15 @@
   </si>
   <si>
     <t>n</t>
+  </si>
+  <si>
+    <t>coke zero</t>
+  </si>
+  <si>
+    <t>coke reg cup</t>
+  </si>
+  <si>
+    <t>coke zero cup</t>
   </si>
 </sst>
 </file>
@@ -640,7 +649,7 @@
         <v>12.7</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="F4" t="s">
         <v>27</v>
@@ -649,7 +658,7 @@
         <v>26</v>
       </c>
       <c r="H4" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="J4" t="s">
         <v>23</v>
@@ -666,7 +675,7 @@
         <v>12.7</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>1.0209999999999999</v>
       </c>
       <c r="F5" t="s">
         <v>27</v>
@@ -675,7 +684,7 @@
         <v>26</v>
       </c>
       <c r="H5" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="J5" t="s">
         <v>23</v>
@@ -692,7 +701,7 @@
         <v>10.9</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F6" t="s">
         <v>28</v>
@@ -718,7 +727,7 @@
         <v>10.9</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F7" t="s">
         <v>28</v>
@@ -744,7 +753,7 @@
         <v>359</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F8" t="s">
         <v>28</v>
@@ -770,7 +779,7 @@
         <v>359</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F9" t="s">
         <v>28</v>
@@ -796,7 +805,7 @@
         <v>359</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F10" t="s">
         <v>28</v>
@@ -822,7 +831,7 @@
         <v>359</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F11" t="s">
         <v>28</v>
@@ -848,7 +857,7 @@
         <v>19.8</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="F12" t="s">
         <v>27</v>
@@ -874,7 +883,7 @@
         <v>19.8</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>1.0209999999999999</v>
       </c>
       <c r="F13" t="s">
         <v>27</v>
@@ -883,7 +892,7 @@
         <v>26</v>
       </c>
       <c r="H13" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="J13" t="s">
         <v>23</v>
@@ -952,7 +961,7 @@
         <v>10.9</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F16" t="s">
         <v>28</v>
@@ -978,7 +987,7 @@
         <v>10.9</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F17" t="s">
         <v>28</v>
@@ -1004,7 +1013,7 @@
         <v>359</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F18" t="s">
         <v>28</v>
@@ -1030,7 +1039,7 @@
         <v>359</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F19" t="s">
         <v>28</v>
@@ -1056,7 +1065,7 @@
         <v>359</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F20" t="s">
         <v>29</v>
@@ -1082,7 +1091,7 @@
         <v>359</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F21" t="s">
         <v>29</v>
@@ -1108,7 +1117,7 @@
         <v>12.7</v>
       </c>
       <c r="D22">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="F22" t="s">
         <v>27</v>
@@ -1117,7 +1126,7 @@
         <v>26</v>
       </c>
       <c r="H22" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="J22" t="s">
         <v>23</v>
@@ -1134,7 +1143,7 @@
         <v>12.7</v>
       </c>
       <c r="D23">
-        <v>1</v>
+        <v>1.0209999999999999</v>
       </c>
       <c r="F23" t="s">
         <v>27</v>
@@ -1143,7 +1152,7 @@
         <v>26</v>
       </c>
       <c r="H23" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="J23" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
added tcn and got good result.
</commit_message>
<xml_diff>
--- a/labeled/june/without straw/Hydrocare_ffinal.xlsx
+++ b/labeled/june/without straw/Hydrocare_ffinal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alireza.mohammadshafie/Documents/hydrocare/labeled/june/without straw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C8BB508-0A09-4042-A575-461ABC9778E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8736B0FD-1C62-254B-90C6-CECF9A0EF457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15100" yWindow="760" windowWidth="15140" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="33">
   <si>
     <t>ID</t>
   </si>
@@ -486,7 +486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC28"/>
+  <dimension ref="A1:AC15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="14.6640625" customWidth="1"/>
@@ -950,323 +950,6 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16">
-        <v>10.9</v>
-      </c>
-      <c r="D16">
-        <v>1.008</v>
-      </c>
-      <c r="F16" t="s">
-        <v>28</v>
-      </c>
-      <c r="G16" t="s">
-        <v>26</v>
-      </c>
-      <c r="H16" t="s">
-        <v>19</v>
-      </c>
-      <c r="J16" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17">
-        <v>10.9</v>
-      </c>
-      <c r="D17">
-        <v>1.008</v>
-      </c>
-      <c r="F17" t="s">
-        <v>28</v>
-      </c>
-      <c r="G17" t="s">
-        <v>26</v>
-      </c>
-      <c r="H17" t="s">
-        <v>19</v>
-      </c>
-      <c r="J17" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18">
-        <v>359</v>
-      </c>
-      <c r="D18">
-        <v>1.008</v>
-      </c>
-      <c r="F18" t="s">
-        <v>28</v>
-      </c>
-      <c r="G18" t="s">
-        <v>26</v>
-      </c>
-      <c r="H18" t="s">
-        <v>22</v>
-      </c>
-      <c r="J18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19">
-        <v>359</v>
-      </c>
-      <c r="D19">
-        <v>1.008</v>
-      </c>
-      <c r="F19" t="s">
-        <v>28</v>
-      </c>
-      <c r="G19" t="s">
-        <v>26</v>
-      </c>
-      <c r="H19" t="s">
-        <v>22</v>
-      </c>
-      <c r="J19" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20">
-        <v>359</v>
-      </c>
-      <c r="D20">
-        <v>1.008</v>
-      </c>
-      <c r="F20" t="s">
-        <v>29</v>
-      </c>
-      <c r="G20" t="s">
-        <v>26</v>
-      </c>
-      <c r="H20" t="s">
-        <v>22</v>
-      </c>
-      <c r="J20" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
-        <v>17</v>
-      </c>
-      <c r="C21">
-        <v>359</v>
-      </c>
-      <c r="D21">
-        <v>1.008</v>
-      </c>
-      <c r="F21" t="s">
-        <v>29</v>
-      </c>
-      <c r="G21" t="s">
-        <v>26</v>
-      </c>
-      <c r="H21" t="s">
-        <v>22</v>
-      </c>
-      <c r="J21" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22">
-        <v>12.7</v>
-      </c>
-      <c r="D22">
-        <v>1.05</v>
-      </c>
-      <c r="F22" t="s">
-        <v>27</v>
-      </c>
-      <c r="G22" t="s">
-        <v>26</v>
-      </c>
-      <c r="H22" t="s">
-        <v>31</v>
-      </c>
-      <c r="J22" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C23">
-        <v>12.7</v>
-      </c>
-      <c r="D23">
-        <v>1.0209999999999999</v>
-      </c>
-      <c r="F23" t="s">
-        <v>27</v>
-      </c>
-      <c r="G23" t="s">
-        <v>26</v>
-      </c>
-      <c r="H23" t="s">
-        <v>32</v>
-      </c>
-      <c r="J23" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24">
-        <v>12.7</v>
-      </c>
-      <c r="D24">
-        <v>1</v>
-      </c>
-      <c r="F24" t="s">
-        <v>29</v>
-      </c>
-      <c r="G24" t="s">
-        <v>26</v>
-      </c>
-      <c r="H24" t="s">
-        <v>21</v>
-      </c>
-      <c r="J24" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25">
-        <v>12.7</v>
-      </c>
-      <c r="D25">
-        <v>1</v>
-      </c>
-      <c r="F25" t="s">
-        <v>29</v>
-      </c>
-      <c r="G25" t="s">
-        <v>26</v>
-      </c>
-      <c r="H25" t="s">
-        <v>21</v>
-      </c>
-      <c r="J25" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26">
-        <v>7.7</v>
-      </c>
-      <c r="D26">
-        <v>1</v>
-      </c>
-      <c r="F26" t="s">
-        <v>29</v>
-      </c>
-      <c r="G26" t="s">
-        <v>26</v>
-      </c>
-      <c r="H26" t="s">
-        <v>20</v>
-      </c>
-      <c r="J26" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27">
-        <v>7.7</v>
-      </c>
-      <c r="D27">
-        <v>1</v>
-      </c>
-      <c r="F27" t="s">
-        <v>29</v>
-      </c>
-      <c r="G27" t="s">
-        <v>26</v>
-      </c>
-      <c r="H27" t="s">
-        <v>20</v>
-      </c>
-      <c r="J27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J28" t="s">
-        <v>23</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>